<commit_message>
Auto-push 2026-05-20T10:09: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase2_Odds_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase2_Odds_Slate.xlsx
@@ -166,32 +166,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-20 05:55:36 ACST</t>
+          <t>2026-05-20 09:56:09 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>flashscore:Uu6uknGb</t>
+          <t>thesportsdb:2475105</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>02:15</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -201,12 +201,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Ajax</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Tottenham</t>
+          <t>Groningen</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -221,67 +221,67 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>10477114</t>
+          <t>10497512</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Ajax</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Tottenham</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>0.7692</t>
+          <t>0.5556</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>0.2381</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>0.0909</t>
+          <t>0.2632</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>1.0982</t>
+          <t>1.0688</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>0.7004</t>
+          <t>0.5198</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>0.2168</t>
+          <t>0.2339</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>0.0828</t>
+          <t>0.2463</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -313,32 +313,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-20 05:55:36 ACST</t>
+          <t>2026-05-20 09:56:09 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>flashscore:rkXMW40U</t>
+          <t>thesportsdb:2475106</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -348,12 +348,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Utrecht</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Manchester City</t>
+          <t>Heerenveen</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -363,97 +363,685 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t/>
+          <t>Sportsbet</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t/>
+          <t>10497513</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t/>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t/>
+          <t>Heerenveen</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t/>
+          <t>1.9</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t/>
+          <t>3.9</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t/>
+          <t>3.5</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t/>
+          <t>0.5263</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t/>
+          <t>0.2564</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t/>
+          <t>0.2857</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t/>
+          <t>1.0684</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t/>
+          <t>0.4926</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t/>
+          <t>0.24</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t/>
+          <t>0.2674</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>thesportsdb:2265408</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>10498423</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2.45</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>0.3636</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>0.2857</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>0.4082</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>1.0575</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0.3438</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>0.2702</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>0.386</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>thesportsdb:2279766</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Celta Vigo</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>10498389</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Celta Vigo</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>4.75</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>0.5714</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>0.2703</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>0.2105</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>1.0522</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0.5431</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>0.2569</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>0.2001</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>thesportsdb:2279764</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Deportivo Alavés</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>unmatched_market</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>No Sportsbet event matched this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>thesportsdb:2279765</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Real Betis</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>10498404</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Betis</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>0.4444</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>0.3077</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>0.303</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>1.0551</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0.4212</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>0.2916</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>0.2872</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>substring</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>0.778</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
         </is>
       </c>
     </row>
@@ -614,32 +1202,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-20 05:55:36 ACST</t>
+          <t>2026-05-20 09:56:09 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>flashscore:Uu6uknGb</t>
+          <t>thesportsdb:2475105</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>02:15</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -649,12 +1237,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Ajax</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Tottenham</t>
+          <t>Groningen</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -669,67 +1257,67 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>10477114</t>
+          <t>10497512</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Ajax</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Tottenham</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>11.0</t>
+          <t>3.8</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>0.7692</t>
+          <t>0.5556</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>0.2381</t>
+          <t>0.25</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>0.0909</t>
+          <t>0.2632</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>1.0982</t>
+          <t>1.0688</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>0.7004</t>
+          <t>0.5198</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>0.2168</t>
+          <t>0.2339</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>0.0828</t>
+          <t>0.2463</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -753,6 +1341,594 @@
         </is>
       </c>
       <c r="AC2" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>thesportsdb:2475106</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Utrecht</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Heerenveen</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>10497513</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>FC Utrecht</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Heerenveen</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>0.5263</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>0.2564</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>0.2857</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>1.0684</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0.4926</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>0.2674</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>thesportsdb:2265408</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>10498423</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2.45</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>0.3636</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>0.2857</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>0.4082</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>1.0575</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0.3438</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>0.2702</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>0.386</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>thesportsdb:2279766</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Celta Vigo</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>10498389</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Celta Vigo</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1.75</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>4.75</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>0.5714</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>0.2703</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>0.2105</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>1.0522</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0.5431</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>0.2569</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>0.2001</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>thesportsdb:2279765</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Real Betis</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>10498404</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Betis</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Levante</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>2.25</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>3.25</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>0.4444</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>0.3077</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>0.303</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>1.0551</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0.4212</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>0.2916</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>0.2872</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>substring</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>0.778</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
         <is>
           <t>Clean Phase 2 odds.</t>
         </is>
@@ -915,32 +2091,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-20 05:55:36 ACST</t>
+          <t>2026-05-20 09:56:09 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>flashscore:rkXMW40U</t>
+          <t>thesportsdb:2279764</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -950,12 +2126,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Deportivo Alavés</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Manchester City</t>
+          <t>Rayo Vallecano</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1270,7 +2446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1280,35 +2456,129 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1371,7 +2641,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-20 05:55:36 ACST</t>
+          <t>2026-05-20 09:56:09 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1381,12 +2651,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>/betting/soccer/united-kingdom/english-premier-league</t>
+          <t>/betting/soccer/rest-of-europe/dutch-eredivisie</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1396,12 +2666,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1410,6 +2680,100 @@
         </is>
       </c>
       <c r="I2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>/betting/soccer/spain/spanish-la-liga</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-20 09:56:09 ACST</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Sportsbet</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>/betting/soccer/italy/italian-serie-a</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1442,7 +2806,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-20 05:55:36 ACST</t>
+          <t>2026-05-20 09:56:09 ACST</t>
         </is>
       </c>
     </row>
@@ -1478,7 +2842,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1490,7 +2854,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1502,7 +2866,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -1514,7 +2878,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ESPN Stats tab and backfill cards/corners from ESPN summary
Phase 1: Expand espn_actuals_for_match() to call /summary endpoint for
yellow+red cards per team; also reads corners from summary as fallback
when scoreboard window is stale. Updates actuals_for() to trigger ESPN
when cards_total is missing, not just corners.

Phase 2: ESPN Stats tab in MatchDetailView. New /api/espn-stats route
proxies scoreboard + summary fetches server-side. EspnStatsSection
renders possession/shots/corners/fouls/cards/saves/offsides bars, key
events timeline, recent form chips, and H2H history. Tab fetches lazily
on first click and resets on match change.

Phase 3: Cache espn_event_id on match dict after first fuzzy name match
so repeat calls (live + results in same run) skip scoreboard scan.
Stub return allows summary-only actuals when event scrolls off window.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase2_Odds_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase2_Odds_Slate.xlsx
@@ -49,115 +49,150 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>timezone</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>home_team_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>home_logo</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>home_goals</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>away</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>away_team_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>away_logo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>away_goals</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
         <is>
           <t>phase1_status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>odds_source</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>sportsbet_event_id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sportsbet_home_name</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>sportsbet_away_name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>home_odds</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>draw_odds</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>away_odds</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>implied_home</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>implied_draw</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>implied_away</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>overround</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>fair_home</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>fair_draw</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>fair_away</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>match_method</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>match_score</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>source_health</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>phase2_status</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>phase2_notes</t>
         </is>
@@ -166,439 +201,362 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 18:58:48 ACST</t>
+          <t>2026-06-17 01:43:32 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>J1 League</t>
+          <t>FIFA World Cup</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>flashscore:fXvLSp0T</t>
+          <t>thesportsdb:2391760</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Machida</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Urawa</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>136516</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://r2.thesportsdb.com/images/media/team/badge/gyfn811591973155.png</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>136143</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://r2.thesportsdb.com/images/media/team/badge/slayb01780546342.png</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>ready_for_phase_2</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t/>
+          <t>Sportsbet</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t/>
+          <t>10425320</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t/>
+          <t>Norway</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t/>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t/>
+          <t>2.15</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t/>
+          <t>3.5</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t/>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>0.4651</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>0.2857</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
+          <t>0.3077</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>1.0585</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>0.4394</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>0.2699</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>0.2907</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
           <t>healthy</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>unmatched_market</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>No Sportsbet event matched this fixture.</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>ready_for_phase_3</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>Clean Phase 2 odds.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-22 18:58:48 ACST</t>
+          <t>2026-06-17 01:43:32 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Allsvenskan</t>
+          <t>FIFA World Cup</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>flashscore:l6SULOIj</t>
+          <t>thesportsdb:2391759</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Djurgarden</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Brommapojkarna</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>140145</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://r2.thesportsdb.com/images/media/team/badge/59fo2s1742100034.png</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>134516</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://r2.thesportsdb.com/images/media/team/badge/rrwpry1455460218.png</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>ready_for_phase_2</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Sportsbet</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>10500468</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Djurgardens</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Brommapojkarna</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>1.4</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>4.6</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>10425306</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>6.5</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>0.7143</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>0.2174</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>0.1538</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>1.0855</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>0.658</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>0.2003</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>0.1417</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>substring</t>
-        </is>
-      </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>0.955</t>
+          <t>0.2439</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
+          <t>0.6667</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>1.0644</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>0.1445</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>0.2291</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0.6264</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
           <t>healthy</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
         <is>
           <t>ready_for_phase_3</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
-        <is>
-          <t>Clean Phase 2 odds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-22 18:58:48 ACST</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Serie A</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>flashscore:ln2VQVwR</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-05-23</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>04:15</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Fiorentina</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Atalanta</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Sportsbet</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>10498423</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Fiorentina</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Atalanta</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>3.4</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>0.3636</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>0.2941</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>1.0577</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>0.3438</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>0.2781</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>0.3782</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>exact</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>ready_for_phase_3</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>Clean Phase 2 odds.</t>
         </is>
@@ -644,115 +602,150 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>timezone</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>home_team_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>home_logo</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>home_goals</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>away</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>away_team_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>away_logo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>away_goals</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
         <is>
           <t>phase1_status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>odds_source</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>sportsbet_event_id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sportsbet_home_name</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>sportsbet_away_name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>home_odds</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>draw_odds</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>away_odds</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>implied_home</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>implied_draw</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>implied_away</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>overround</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>fair_home</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>fair_draw</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>fair_away</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>match_method</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>match_score</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>source_health</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>phase2_status</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>phase2_notes</t>
         </is>
@@ -761,145 +754,180 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 18:58:48 ACST</t>
+          <t>2026-06-17 01:43:32 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Allsvenskan</t>
+          <t>FIFA World Cup</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>flashscore:l6SULOIj</t>
+          <t>thesportsdb:2391760</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Djurgarden</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Brommapojkarna</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>136516</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>https://r2.thesportsdb.com/images/media/team/badge/gyfn811591973155.png</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>136143</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://r2.thesportsdb.com/images/media/team/badge/slayb01780546342.png</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>ready_for_phase_2</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Sportsbet</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>10500468</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Djurgardens</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Brommapojkarna</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>1.4</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>4.6</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>0.7143</t>
-        </is>
-      </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>0.2174</t>
+          <t>10425320</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>0.1538</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>1.0855</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>0.658</t>
+          <t>2.15</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>0.2003</t>
+          <t>3.5</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>0.1417</t>
+          <t>3.25</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>substring</t>
+          <t>0.4651</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>0.955</t>
+          <t>0.2857</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
+          <t>0.3077</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>1.0585</t>
+        </is>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>0.4394</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>0.2699</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>0.2907</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="AH2" t="inlineStr">
+        <is>
           <t>healthy</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>ready_for_phase_3</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>Clean Phase 2 odds.</t>
         </is>
@@ -908,145 +936,180 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-22 18:58:48 ACST</t>
+          <t>2026-06-17 01:43:32 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>FIFA World Cup</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>flashscore:ln2VQVwR</t>
+          <t>thesportsdb:2391759</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Fiorentina</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>140145</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://r2.thesportsdb.com/images/media/team/badge/59fo2s1742100034.png</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>134516</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://r2.thesportsdb.com/images/media/team/badge/rrwpry1455460218.png</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>ready_for_phase_2</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Sportsbet</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>10498423</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Fiorentina</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Atalanta</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>3.4</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>0.3636</t>
-        </is>
-      </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>0.2941</t>
+          <t>10425306</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>1.0577</t>
+          <t>Algeria</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>0.3438</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>0.2781</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>0.3782</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
+          <t>0.1538</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>0.2439</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>0.6667</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>1.0644</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>0.1445</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>0.2291</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0.6264</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
           <t>exact</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>1.0</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AH3" t="inlineStr">
         <is>
           <t>healthy</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
         <is>
           <t>ready_for_phase_3</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>Clean Phase 2 odds.</t>
         </is>
@@ -1092,264 +1155,152 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>timezone</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>home_team_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>home_logo</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>home_goals</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>away</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>away_team_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>away_logo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>away_goals</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
         <is>
           <t>phase1_status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>odds_source</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>sportsbet_event_id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sportsbet_home_name</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>sportsbet_away_name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>home_odds</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>draw_odds</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>away_odds</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>implied_home</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>implied_draw</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>implied_away</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>overround</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>fair_home</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>fair_draw</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>fair_away</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>match_method</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>match_score</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>source_health</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>phase2_status</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>phase2_notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-05-22 18:58:48 ACST</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>196</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>J1 League</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>flashscore:fXvLSp0T</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Machida</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Urawa</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>unmatched_market</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>No Sportsbet event matched this fixture.</t>
         </is>
       </c>
     </row>
@@ -1393,115 +1344,150 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>timezone</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>home_team_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>home_logo</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>home_goals</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
         <is>
           <t>away</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>away_team_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>away_logo</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>away_goals</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
         <is>
           <t>phase1_status</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>odds_source</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>sportsbet_event_id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sportsbet_home_name</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>sportsbet_away_name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>home_odds</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>draw_odds</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>away_odds</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>implied_home</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>implied_draw</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>implied_away</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>overround</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>fair_home</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>fair_draw</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>fair_away</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>match_method</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>match_score</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>source_health</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>phase2_status</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>phase2_notes</t>
         </is>
@@ -1564,17 +1550,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Allsvenskan</t>
+          <t>FIFA World Cup</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1603,100 +1589,6 @@
         </is>
       </c>
       <c r="I2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>J1 League</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Serie A</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1759,7 +1651,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 18:58:48 ACST</t>
+          <t>2026-06-17 01:43:32 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1769,12 +1661,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Allsvenskan</t>
+          <t>FIFA World Cup</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>/betting/soccer/rest-of-europe/swedish-allsvenskan</t>
+          <t>/betting/soccer/world-cup/mens-world-cup</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1784,12 +1676,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>56</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>56</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1798,100 +1690,6 @@
         </is>
       </c>
       <c r="I2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-22 18:58:48 ACST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Sportsbet</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>J1 League</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>/betting/soccer/asia/japanese-j1-league</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-22 18:58:48 ACST</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Sportsbet</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Serie A</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>/betting/soccer/italy/italian-serie-a</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
         <is>
           <t/>
         </is>
@@ -1924,7 +1722,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-22 18:58:48 ACST</t>
+          <t>2026-06-17 01:43:32 ACST</t>
         </is>
       </c>
     </row>
@@ -1955,43 +1753,43 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>phase1_input_rows</t>
+          <t>target_dates</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2026-06-23</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>phase1_ready_rows</t>
+          <t>phase1_input_rows</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>phase2_total_rows</t>
+          <t>phase1_ready_rows</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ready_for_phase_3</t>
+          <t>phase2_total_rows</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2003,19 +1801,19 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>unmatched_market</t>
+          <t>ready_for_phase_3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>partial_market</t>
+          <t>unmatched_market</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2027,7 +1825,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>implausible_overround</t>
+          <t>partial_market</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2039,7 +1837,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>low_match_confidence</t>
+          <t>implausible_overround</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2051,7 +1849,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>source_blocked</t>
+          <t>low_match_confidence</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2063,7 +1861,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>upstream_blocked</t>
+          <t>source_blocked</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2075,10 +1873,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>upstream_blocked</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>next_action</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Proceed with Phase 3 for ready_for_phase_3 rows.</t>
         </is>

</xml_diff>